<commit_message>
fix(excel): IF(INPUT!Dx5="","",INPUT!Dx5) evite 0 dans RATIOS/DCF, synthese effacee MC.PA
</commit_message>
<xml_diff>
--- a/assets/TEMPLATE.xlsx
+++ b/assets/TEMPLATE.xlsx
@@ -11514,23 +11514,23 @@
       </c>
       <c r="C5" s="1" t="n"/>
       <c r="D5" s="1">
-        <f>INPUT!D5</f>
+        <f>IF(INPUT!D5="","",INPUT!D5)</f>
         <v/>
       </c>
       <c r="E5" s="1">
-        <f>INPUT!E5</f>
+        <f>IF(INPUT!E5="","",INPUT!E5)</f>
         <v/>
       </c>
       <c r="F5" s="1">
-        <f>INPUT!F5</f>
+        <f>IF(INPUT!F5="","",INPUT!F5)</f>
         <v/>
       </c>
       <c r="G5" s="1">
-        <f>INPUT!G5</f>
+        <f>IF(INPUT!G5="","",INPUT!G5)</f>
         <v/>
       </c>
       <c r="H5" s="1">
-        <f>INPUT!H5</f>
+        <f>IF(INPUT!H5="","",INPUT!H5)</f>
         <v/>
       </c>
     </row>
@@ -13778,23 +13778,23 @@
       </c>
       <c r="C5" s="138" t="n"/>
       <c r="D5" s="138">
-        <f>INPUT!D5</f>
+        <f>IF(INPUT!D5="","",INPUT!D5)</f>
         <v/>
       </c>
       <c r="E5" s="138">
-        <f>INPUT!E5</f>
+        <f>IF(INPUT!E5="","",INPUT!E5)</f>
         <v/>
       </c>
       <c r="F5" s="138">
-        <f>INPUT!F5</f>
+        <f>IF(INPUT!F5="","",INPUT!F5)</f>
         <v/>
       </c>
       <c r="G5" s="138">
-        <f>INPUT!G5</f>
+        <f>IF(INPUT!G5="","",INPUT!G5)</f>
         <v/>
       </c>
       <c r="H5" s="138">
-        <f>INPUT!H5</f>
+        <f>IF(INPUT!H5="","",INPUT!H5)</f>
         <v/>
       </c>
       <c r="I5" s="24" t="n"/>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="E5" s="16">
-        <f>INPUT!H5</f>
+        <f>IF(INPUT!H5="","",INPUT!H5)</f>
         <v/>
       </c>
       <c r="F5" s="16" t="inlineStr">
@@ -16258,23 +16258,23 @@
         </is>
       </c>
       <c r="D5" s="24">
-        <f>INPUT!D5</f>
+        <f>IF(INPUT!D5="","",INPUT!D5)</f>
         <v/>
       </c>
       <c r="E5" s="24">
-        <f>INPUT!E5</f>
+        <f>IF(INPUT!E5="","",INPUT!E5)</f>
         <v/>
       </c>
       <c r="F5" s="24">
-        <f>INPUT!F5</f>
+        <f>IF(INPUT!F5="","",INPUT!F5)</f>
         <v/>
       </c>
       <c r="G5" s="24">
-        <f>INPUT!G5</f>
+        <f>IF(INPUT!G5="","",INPUT!G5)</f>
         <v/>
       </c>
       <c r="H5" s="24">
-        <f>INPUT!H5</f>
+        <f>IF(INPUT!H5="","",INPUT!H5)</f>
         <v/>
       </c>
       <c r="I5" s="24">

</xml_diff>

<commit_message>
fix(pptx+excel): slide 16/18 bugs, Dashboard CF colonnes vides
PPTX:
- slide 16: _truncate 370->480 chars (counter_thesis ~380 chars evitait le "...")
- slide 18: themes table = 1er theme seulement (evite expansion hauteur),
  comment_y = max(calc, 11.5cm) pour eviter chevauchement definitif

Excel TEMPLATE.xlsx:
- CF hide-empty-col sur DASHBOARD 2 (cols T-X = annees D-H)
- CF hide-empty-col sur DASHBOARD (cols C, D-H, J-N)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/TEMPLATE.xlsx
+++ b/assets/TEMPLATE.xlsx
@@ -25589,6 +25589,61 @@
     <brk id="41" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <conditionalFormatting sqref="C1:C200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>INPUT!$F$128&lt;5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D200">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>INPUT!$F$128&lt;5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E1:E200">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>INPUT!$F$128&lt;4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F1:F200">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>INPUT!$F$128&lt;3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:G200">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>INPUT!$F$128&lt;2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:H200">
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>INPUT!$F$128&lt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J1:J200">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>INPUT!$F$128&lt;5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K1:K200">
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>INPUT!$F$128&lt;4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L1:L200">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>INPUT!$F$128&lt;3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M1:M200">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>INPUT!$F$128&lt;2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N1:N200">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>INPUT!$F$128&lt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
 
@@ -28168,5 +28223,30 @@
   <pageMargins left="0.005555555555555556" right="0.005555555555555556" top="0.005555555555555556" bottom="0.005555555555555556" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <conditionalFormatting sqref="T1:T200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>INPUT!$F$128&lt;5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U1:U200">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>INPUT!$F$128&lt;4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V1:V200">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>INPUT!$F$128&lt;3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W1:W200">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>INPUT!$F$128&lt;2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X1:X200">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>INPUT!$F$128&lt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
</xml_diff>